<commit_message>
chore: deploy refreshed floor fixtures
</commit_message>
<xml_diff>
--- a/fixtures/fp-tests/3.xlsx
+++ b/fixtures/fp-tests/3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft3248279.sharepoint.com/sites/asseticom/Shared Documents/General/04. Software Services/02. Live/C&amp;B - Equans Life Cycle Surveys/North Lanarkshire Schools/Data Imports M&amp;E/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexstanbury/Downloads/FP_Tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C95B3D63-4985-44F6-B0F0-B3A837B125B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66250AEC-6EA8-DC40-8C53-530E947AD791}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{90C03551-7412-466B-B1C1-5284A9DECD66}"/>
+    <workbookView xWindow="28680" yWindow="600" windowWidth="29040" windowHeight="15840" xr2:uid="{90C03551-7412-466B-B1C1-5284A9DECD66}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="116">
   <si>
     <t>Floor</t>
   </si>
@@ -387,12 +387,6 @@
   </si>
   <si>
     <t>G21E - WC</t>
-  </si>
-  <si>
-    <t>Whole Building</t>
-  </si>
-  <si>
-    <t>THROUGHOUT</t>
   </si>
 </sst>
 </file>
@@ -786,14 +780,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A51B8E68-E7D8-4616-9586-3249837F8B28}">
-  <dimension ref="A1:D113"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D112"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.21875" customWidth="1"/>
-    <col min="2" max="2" width="50.109375" customWidth="1"/>
+    <col min="1" max="1" width="18.1640625" customWidth="1"/>
+    <col min="2" max="2" width="50.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -807,7 +801,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -821,7 +815,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -835,7 +829,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -849,7 +843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -863,7 +857,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -877,7 +871,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -891,7 +885,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -905,7 +899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -919,7 +913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -933,7 +927,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -947,7 +941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -961,7 +955,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -975,7 +969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -989,7 +983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -1003,7 +997,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>4</v>
       </c>
@@ -1017,7 +1011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>4</v>
       </c>
@@ -1031,7 +1025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>4</v>
       </c>
@@ -1045,7 +1039,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>4</v>
       </c>
@@ -1059,7 +1053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>4</v>
       </c>
@@ -1073,7 +1067,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>4</v>
       </c>
@@ -1087,7 +1081,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>4</v>
       </c>
@@ -1101,7 +1095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>4</v>
       </c>
@@ -1115,7 +1109,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>4</v>
       </c>
@@ -1129,7 +1123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>4</v>
       </c>
@@ -1143,7 +1137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>4</v>
       </c>
@@ -1157,7 +1151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>4</v>
       </c>
@@ -1171,7 +1165,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>4</v>
       </c>
@@ -1185,7 +1179,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>4</v>
       </c>
@@ -1199,7 +1193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>4</v>
       </c>
@@ -1213,7 +1207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>4</v>
       </c>
@@ -1227,7 +1221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>4</v>
       </c>
@@ -1241,7 +1235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>4</v>
       </c>
@@ -1255,7 +1249,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>4</v>
       </c>
@@ -1269,7 +1263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>4</v>
       </c>
@@ -1283,7 +1277,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>4</v>
       </c>
@@ -1297,7 +1291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>4</v>
       </c>
@@ -1311,7 +1305,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>4</v>
       </c>
@@ -1325,7 +1319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>4</v>
       </c>
@@ -1339,7 +1333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>4</v>
       </c>
@@ -1353,7 +1347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>4</v>
       </c>
@@ -1367,7 +1361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>4</v>
       </c>
@@ -1381,7 +1375,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>4</v>
       </c>
@@ -1395,7 +1389,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>4</v>
       </c>
@@ -1409,7 +1403,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>4</v>
       </c>
@@ -1423,7 +1417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>4</v>
       </c>
@@ -1437,7 +1431,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>4</v>
       </c>
@@ -1451,7 +1445,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>4</v>
       </c>
@@ -1465,7 +1459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>4</v>
       </c>
@@ -1479,7 +1473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>4</v>
       </c>
@@ -1493,7 +1487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>4</v>
       </c>
@@ -1507,7 +1501,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>4</v>
       </c>
@@ -1521,7 +1515,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>4</v>
       </c>
@@ -1535,7 +1529,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>4</v>
       </c>
@@ -1549,7 +1543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>4</v>
       </c>
@@ -1563,7 +1557,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>4</v>
       </c>
@@ -1577,7 +1571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>4</v>
       </c>
@@ -1591,7 +1585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>4</v>
       </c>
@@ -1605,7 +1599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>4</v>
       </c>
@@ -1619,7 +1613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>4</v>
       </c>
@@ -1633,7 +1627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>4</v>
       </c>
@@ -1647,7 +1641,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>4</v>
       </c>
@@ -1661,7 +1655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>4</v>
       </c>
@@ -1675,7 +1669,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>4</v>
       </c>
@@ -1689,7 +1683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>4</v>
       </c>
@@ -1703,7 +1697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>4</v>
       </c>
@@ -1717,7 +1711,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>4</v>
       </c>
@@ -1731,7 +1725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>4</v>
       </c>
@@ -1745,7 +1739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>4</v>
       </c>
@@ -1759,7 +1753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>4</v>
       </c>
@@ -1773,7 +1767,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>4</v>
       </c>
@@ -1787,7 +1781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>4</v>
       </c>
@@ -1801,7 +1795,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>4</v>
       </c>
@@ -1815,7 +1809,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>4</v>
       </c>
@@ -1829,7 +1823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>4</v>
       </c>
@@ -1843,7 +1837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>4</v>
       </c>
@@ -1857,7 +1851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>4</v>
       </c>
@@ -1871,7 +1865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>4</v>
       </c>
@@ -1885,7 +1879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>4</v>
       </c>
@@ -1899,7 +1893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>4</v>
       </c>
@@ -1913,7 +1907,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>4</v>
       </c>
@@ -1927,7 +1921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>4</v>
       </c>
@@ -1941,7 +1935,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>4</v>
       </c>
@@ -1955,7 +1949,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>4</v>
       </c>
@@ -1969,7 +1963,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>4</v>
       </c>
@@ -1983,7 +1977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>4</v>
       </c>
@@ -1997,7 +1991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>4</v>
       </c>
@@ -2011,7 +2005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>4</v>
       </c>
@@ -2025,7 +2019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>4</v>
       </c>
@@ -2039,7 +2033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>4</v>
       </c>
@@ -2053,7 +2047,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>4</v>
       </c>
@@ -2067,7 +2061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>4</v>
       </c>
@@ -2081,7 +2075,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>4</v>
       </c>
@@ -2095,7 +2089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>4</v>
       </c>
@@ -2109,7 +2103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>4</v>
       </c>
@@ -2123,7 +2117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>4</v>
       </c>
@@ -2137,7 +2131,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>4</v>
       </c>
@@ -2151,7 +2145,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>4</v>
       </c>
@@ -2165,7 +2159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>4</v>
       </c>
@@ -2179,7 +2173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>4</v>
       </c>
@@ -2193,7 +2187,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>4</v>
       </c>
@@ -2207,7 +2201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>4</v>
       </c>
@@ -2221,7 +2215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>4</v>
       </c>
@@ -2235,7 +2229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>4</v>
       </c>
@@ -2249,7 +2243,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>4</v>
       </c>
@@ -2263,7 +2257,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>4</v>
       </c>
@@ -2277,7 +2271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>4</v>
       </c>
@@ -2291,7 +2285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>4</v>
       </c>
@@ -2305,7 +2299,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>4</v>
       </c>
@@ -2319,7 +2313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>4</v>
       </c>
@@ -2333,7 +2327,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>4</v>
       </c>
@@ -2347,7 +2341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>4</v>
       </c>
@@ -2359,14 +2353,6 @@
       </c>
       <c r="D112">
         <v>0</v>
-      </c>
-    </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A113" t="s">
-        <v>116</v>
-      </c>
-      <c r="B113" t="s">
-        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -2376,6 +2362,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="5db48b64-35f6-4468-8f7d-90ba9a0a6b12" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="28abb233-3e57-4edf-8235-d6ecf6a0ac5a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_x0032_026 xmlns="28abb233-3e57-4edf-8235-d6ecf6a0ac5a">false</_x0032_026>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000540BAE173F065488F2BDC1098F32ACD" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c1ca55ac7cba354ca8a599c61de167ef">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="28abb233-3e57-4edf-8235-d6ecf6a0ac5a" xmlns:ns3="5db48b64-35f6-4468-8f7d-90ba9a0a6b12" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd828bd328a808308cf08e1b855890b0" ns2:_="" ns3:_="">
     <xsd:import namespace="28abb233-3e57-4edf-8235-d6ecf6a0ac5a"/>
@@ -2622,35 +2629,40 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="5db48b64-35f6-4468-8f7d-90ba9a0a6b12" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="28abb233-3e57-4edf-8235-d6ecf6a0ac5a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_x0032_026 xmlns="28abb233-3e57-4edf-8235-d6ecf6a0ac5a">false</_x0032_026>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{388C0A14-D03F-4E29-9182-F2D1EF0CBF84}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{96D44A0D-D244-4972-8705-2AB7788FD882}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="5db48b64-35f6-4468-8f7d-90ba9a0a6b12"/>
+    <ds:schemaRef ds:uri="28abb233-3e57-4edf-8235-d6ecf6a0ac5a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AF05D756-19C4-4AE2-A1DE-2963B56798D2}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AF05D756-19C4-4AE2-A1DE-2963B56798D2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{96D44A0D-D244-4972-8705-2AB7788FD882}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{388C0A14-D03F-4E29-9182-F2D1EF0CBF84}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="28abb233-3e57-4edf-8235-d6ecf6a0ac5a"/>
+    <ds:schemaRef ds:uri="5db48b64-35f6-4468-8f7d-90ba9a0a6b12"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>